<commit_message>
Sincronizar el espejo: 1.932 laminas y payloads al dia
El espejo venia quedandose atras, y eso hacia visibles dos cosas ya
corregidas aguas arriba:

- Los cuatro indicadores demograficos comunales mostraban las tarjetas
  "Valor regional" y "Valor nacional" vacias. El bug se corrigio el
  2026-09-01 en generate_comunal_mapa.R: esos indicadores leen
  demograficos_comunal_anual.csv, que trae SOLO el nivel comuna, y hacia
  falta un puente que redirija archivo Y codigo a la vez (D_ENV_a ->
  D_ENVEJE_a en demografia_indicadores_anual.csv). Las laminas corregidas
  nunca habian llegado a este repo.

- Entre 2018 y 2022, Aysen mostraba las cifras de Valparaiso en los cinco
  indicadores demograficos (ver PIDR c9bf928f). Van las laminas regeneradas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nb4kJtgDC9tzWdETyfNewy
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_nacional_d_deptot_a_2018.xlsx
+++ b/output/graficos_nacionales/plot_nacional_d_deptot_a_2018.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="730">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -2161,7 +2161,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-27 21:56</t>
+    <t xml:space="preserve">2026-09-04 19:37</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -2173,16 +2173,25 @@
     <t xml:space="preserve">Imagen asociada</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
+    <t xml:space="preserve">plot_nacional_d_deptot_a_2018.png</t>
   </si>
   <si>
     <t xml:space="preserve">Indicador</t>
   </si>
   <si>
+    <t xml:space="preserve">Dependencia demográfica total</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unidad territorial</t>
   </si>
   <si>
+    <t xml:space="preserve">Comuna (vista nacional macrozonal)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018</t>
   </si>
   <si>
     <t xml:space="preserve">variable</t>
@@ -13571,23 +13580,23 @@
         <v>719</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
   </sheetData>
@@ -13609,21 +13618,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
@@ -13632,7 +13641,7 @@
         <v>2018</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>

</xml_diff>